<commit_message>
Q325 Earnings Season pt.1
</commit_message>
<xml_diff>
--- a/Financial Analysis/AMD.xlsx
+++ b/Financial Analysis/AMD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antos\Documents\GitHub\FinanceModels\Financial Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90592336-7628-436E-A184-C7AEEF03C703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0662FF93-B5FE-4FBE-A730-15236FEF286B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9151AF15-9D45-44A9-8CA3-26C538A98864}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{9151AF15-9D45-44A9-8CA3-26C538A98864}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -232,10 +232,10 @@
     <t>Restructuring</t>
   </si>
   <si>
-    <t>Q225 8K</t>
-  </si>
-  <si>
-    <t>Slightly undervalued</t>
+    <t>Slightly overvalued</t>
+  </si>
+  <si>
+    <t>Q325 8K</t>
   </si>
 </sst>
 </file>
@@ -335,14 +335,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
@@ -359,7 +359,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13106400" y="0"/>
+          <a:off x="13708380" y="0"/>
           <a:ext cx="0" cy="6499860"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -759,17 +759,17 @@
         <v>1</v>
       </c>
       <c r="D3" s="4">
-        <v>150.74</v>
+        <v>239.23</v>
       </c>
       <c r="E3" s="2">
-        <v>45918</v>
+        <v>45966</v>
       </c>
       <c r="F3" s="2">
         <f ca="1">TODAY()</f>
-        <v>45918</v>
+        <v>45966</v>
       </c>
       <c r="G3" s="2">
-        <v>45967</v>
+        <v>46056</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
@@ -777,11 +777,11 @@
         <v>2</v>
       </c>
       <c r="D4" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
@@ -790,7 +790,7 @@
       </c>
       <c r="D5" s="5">
         <f>D3*D4</f>
-        <v>244651.02000000002</v>
+        <v>388987.98</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
@@ -798,11 +798,11 @@
         <v>4</v>
       </c>
       <c r="D6" s="5">
-        <f>4442+1425</f>
-        <v>5867</v>
+        <f>4808+2435</f>
+        <v>7243</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
@@ -810,11 +810,11 @@
         <v>5</v>
       </c>
       <c r="D7" s="5">
-        <f>3218</f>
-        <v>3218</v>
+        <f>873+2347</f>
+        <v>3220</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
@@ -823,7 +823,7 @@
       </c>
       <c r="D8" s="5">
         <f>D6-D7</f>
-        <v>2649</v>
+        <v>4023</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
@@ -832,7 +832,7 @@
       </c>
       <c r="D9" s="5">
         <f>D5-D8</f>
-        <v>242002.02000000002</v>
+        <v>384964.98</v>
       </c>
     </row>
   </sheetData>
@@ -1024,11 +1024,11 @@
         <v>7685</v>
       </c>
       <c r="U3" s="8">
-        <v>8700</v>
+        <v>9246</v>
       </c>
       <c r="V3" s="8">
-        <f>R3*1.25</f>
-        <v>9572.5</v>
+        <f>R3*1.27</f>
+        <v>9725.66</v>
       </c>
       <c r="Y3" s="8">
         <v>6731</v>
@@ -1053,47 +1053,47 @@
       </c>
       <c r="AE3" s="8">
         <f>SUM(S3:V3)</f>
-        <v>33395.5</v>
+        <v>34094.660000000003</v>
       </c>
       <c r="AF3" s="8">
-        <f>AE3*1.2</f>
-        <v>40074.6</v>
+        <f>AE3*1.23</f>
+        <v>41936.431800000006</v>
       </c>
       <c r="AG3" s="8">
         <f>AF3*1.15</f>
-        <v>46085.789999999994</v>
+        <v>48226.896570000004</v>
       </c>
       <c r="AH3" s="8">
         <f>AG3*1.1</f>
-        <v>50694.368999999999</v>
+        <v>53049.586227000007</v>
       </c>
       <c r="AI3" s="8">
         <f>AH3*1.09</f>
-        <v>55256.862209999999</v>
+        <v>57824.048987430011</v>
       </c>
       <c r="AJ3" s="8">
         <f>AI3*1.07</f>
-        <v>59124.842564700004</v>
+        <v>61871.732416550112</v>
       </c>
       <c r="AK3" s="8">
         <f>AJ3*1.05</f>
-        <v>62081.084692935008</v>
+        <v>64965.319037377623</v>
       </c>
       <c r="AL3" s="8">
         <f t="shared" ref="AL3:AO3" si="0">AK3*1.05</f>
-        <v>65185.138927581764</v>
+        <v>68213.584989246505</v>
       </c>
       <c r="AM3" s="8">
         <f t="shared" si="0"/>
-        <v>68444.39587396085</v>
+        <v>71624.264238708827</v>
       </c>
       <c r="AN3" s="8">
         <f t="shared" si="0"/>
-        <v>71866.615667658902</v>
+        <v>75205.477450644277</v>
       </c>
       <c r="AO3" s="8">
         <f t="shared" si="0"/>
-        <v>75459.946451041847</v>
+        <v>78965.75132317649</v>
       </c>
     </row>
     <row r="4" spans="2:41" x14ac:dyDescent="0.3">
@@ -1155,8 +1155,13 @@
       <c r="T4" s="5">
         <v>4366</v>
       </c>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
+      <c r="U4" s="5">
+        <v>4206</v>
+      </c>
+      <c r="V4" s="5">
+        <f>V6-V5</f>
+        <v>4155.1752999999999</v>
+      </c>
       <c r="Y4" s="5">
         <v>3863</v>
       </c>
@@ -1178,7 +1183,10 @@
         <f>SUM(O4:R4)</f>
         <v>12114</v>
       </c>
-      <c r="AE4" s="5"/>
+      <c r="AE4" s="5">
+        <f>SUM(S4:V4)</f>
+        <v>16178.175299999999</v>
+      </c>
       <c r="AF4" s="5"/>
       <c r="AG4" s="5"/>
       <c r="AH4" s="5"/>
@@ -1249,8 +1257,12 @@
       <c r="T5" s="5">
         <v>260</v>
       </c>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
+      <c r="U5" s="5">
+        <v>260</v>
+      </c>
+      <c r="V5" s="5">
+        <v>270</v>
+      </c>
       <c r="Y5" s="5"/>
       <c r="Z5" s="5"/>
       <c r="AA5" s="5"/>
@@ -1266,7 +1278,10 @@
         <f>SUM(O5:R5)</f>
         <v>946</v>
       </c>
-      <c r="AE5" s="5"/>
+      <c r="AE5" s="5">
+        <f>SUM(S5:V5)</f>
+        <v>1041</v>
+      </c>
       <c r="AF5" s="5"/>
       <c r="AG5" s="5"/>
       <c r="AH5" s="5"/>
@@ -1283,7 +1298,7 @@
         <v>16</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" ref="C6:T6" si="1">SUM(C4:C5)</f>
+        <f t="shared" ref="C6:U6" si="1">SUM(C4:C5)</f>
         <v>1858</v>
       </c>
       <c r="D6" s="5">
@@ -1355,12 +1370,12 @@
         <v>4626</v>
       </c>
       <c r="U6" s="5">
-        <f t="shared" ref="U6:V6" si="2">U3-U7</f>
-        <v>4089</v>
+        <f t="shared" si="1"/>
+        <v>4466</v>
       </c>
       <c r="V6" s="5">
-        <f t="shared" si="2"/>
-        <v>4403.3499999999995</v>
+        <f t="shared" ref="V6" si="2">V3-V7</f>
+        <v>4425.1752999999999</v>
       </c>
       <c r="Y6" s="5">
         <f t="shared" ref="Y6:AD6" si="3">SUM(Y4:Y5)</f>
@@ -1388,47 +1403,47 @@
       </c>
       <c r="AE6" s="5">
         <f>SUM(S6:V6)</f>
-        <v>16820.349999999999</v>
+        <v>17219.175299999999</v>
       </c>
       <c r="AF6" s="5">
         <f>AF3-AF7</f>
-        <v>18033.569999999996</v>
+        <v>18871.39431</v>
       </c>
       <c r="AG6" s="5">
         <f t="shared" ref="AG6:AO6" si="4">AG3-AG7</f>
-        <v>19816.8897</v>
+        <v>20737.565525100003</v>
       </c>
       <c r="AH6" s="5">
         <f t="shared" si="4"/>
-        <v>20784.691290000002</v>
+        <v>22280.826215340006</v>
       </c>
       <c r="AI6" s="5">
         <f t="shared" si="4"/>
-        <v>22102.744884</v>
+        <v>23707.860084846303</v>
       </c>
       <c r="AJ6" s="5">
         <f t="shared" si="4"/>
-        <v>23058.688600232999</v>
+        <v>24748.692966620045</v>
       </c>
       <c r="AK6" s="5">
         <f t="shared" si="4"/>
-        <v>23590.812183315305</v>
+        <v>25986.127614951052</v>
       </c>
       <c r="AL6" s="5">
         <f t="shared" si="4"/>
-        <v>24770.35279248107</v>
+        <v>27285.4339956986</v>
       </c>
       <c r="AM6" s="5">
         <f t="shared" si="4"/>
-        <v>26008.870432105126</v>
+        <v>28649.705695483535</v>
       </c>
       <c r="AN6" s="5">
         <f t="shared" si="4"/>
-        <v>27309.313953710385</v>
+        <v>30082.190980257714</v>
       </c>
       <c r="AO6" s="5">
         <f t="shared" si="4"/>
-        <v>28674.779651395904</v>
+        <v>31586.3005292706</v>
       </c>
     </row>
     <row r="7" spans="2:41" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1436,7 +1451,7 @@
         <v>18</v>
       </c>
       <c r="C7" s="8">
-        <f t="shared" ref="C7:T7" si="5">C3-C6</f>
+        <f t="shared" ref="C7:U7" si="5">C3-C6</f>
         <v>1587</v>
       </c>
       <c r="D7" s="8">
@@ -1508,12 +1523,12 @@
         <v>3059</v>
       </c>
       <c r="U7" s="8">
-        <f>U3*0.53</f>
-        <v>4611</v>
+        <f t="shared" si="5"/>
+        <v>4780</v>
       </c>
       <c r="V7" s="8">
-        <f>V3*0.54</f>
-        <v>5169.1500000000005</v>
+        <f>V3*0.545</f>
+        <v>5300.4847</v>
       </c>
       <c r="Y7" s="8">
         <f t="shared" ref="Y7:AE7" si="6">Y3-Y6</f>
@@ -1541,47 +1556,47 @@
       </c>
       <c r="AE7" s="8">
         <f t="shared" si="6"/>
-        <v>16575.150000000001</v>
+        <v>16875.484700000005</v>
       </c>
       <c r="AF7" s="8">
         <f>AF3*0.55</f>
-        <v>22041.030000000002</v>
+        <v>23065.037490000006</v>
       </c>
       <c r="AG7" s="8">
         <f>AG3*0.57</f>
-        <v>26268.900299999994</v>
+        <v>27489.331044900002</v>
       </c>
       <c r="AH7" s="8">
-        <f>AH3*0.59</f>
-        <v>29909.677709999996</v>
+        <f>AH3*0.58</f>
+        <v>30768.760011660001</v>
       </c>
       <c r="AI7" s="8">
-        <f>AI3*0.6</f>
-        <v>33154.117326</v>
+        <f>AI3*0.59</f>
+        <v>34116.188902583708</v>
       </c>
       <c r="AJ7" s="8">
-        <f>AJ3*0.61</f>
-        <v>36066.153964467005</v>
+        <f>AJ3*0.6</f>
+        <v>37123.039449930067</v>
       </c>
       <c r="AK7" s="8">
-        <f>AK3*0.62</f>
-        <v>38490.272509619703</v>
+        <f t="shared" ref="AK7:AO7" si="7">AK3*0.6</f>
+        <v>38979.191422426571</v>
       </c>
       <c r="AL7" s="8">
-        <f t="shared" ref="AL7:AO7" si="7">AL3*0.62</f>
-        <v>40414.786135100694</v>
+        <f t="shared" si="7"/>
+        <v>40928.150993547904</v>
       </c>
       <c r="AM7" s="8">
         <f t="shared" si="7"/>
-        <v>42435.525441855723</v>
+        <v>42974.558543225292</v>
       </c>
       <c r="AN7" s="8">
         <f t="shared" si="7"/>
-        <v>44557.301713948516</v>
+        <v>45123.286470386563</v>
       </c>
       <c r="AO7" s="8">
         <f t="shared" si="7"/>
-        <v>46785.166799645944</v>
+        <v>47379.450793905889</v>
       </c>
     </row>
     <row r="8" spans="2:41" x14ac:dyDescent="0.3">
@@ -1644,12 +1659,11 @@
         <v>1894</v>
       </c>
       <c r="U8" s="5">
-        <f>Q8*1.22</f>
-        <v>1995.9199999999998</v>
+        <v>2139</v>
       </c>
       <c r="V8" s="5">
-        <f>R8*1.2</f>
-        <v>2054.4</v>
+        <f>R8*1.28</f>
+        <v>2191.36</v>
       </c>
       <c r="Y8" s="5">
         <v>1547</v>
@@ -1674,47 +1688,47 @@
       </c>
       <c r="AE8" s="5">
         <f>SUM(S8:V8)</f>
-        <v>7672.32</v>
+        <v>7952.3600000000006</v>
       </c>
       <c r="AF8" s="5">
-        <f>AE8*1.13</f>
-        <v>8669.7215999999989</v>
+        <f>AE8*1.14</f>
+        <v>9065.6903999999995</v>
       </c>
       <c r="AG8" s="5">
         <f>AF8*1.08</f>
-        <v>9363.2993279999992</v>
+        <v>9790.9456320000008</v>
       </c>
       <c r="AH8" s="5">
         <f>AG8*1.06</f>
-        <v>9925.0972876799988</v>
+        <v>10378.402369920001</v>
       </c>
       <c r="AI8" s="5">
         <f>AH8*1.04</f>
-        <v>10322.101179187199</v>
+        <v>10793.538464716801</v>
       </c>
       <c r="AJ8" s="5">
         <f>AI8*1.03</f>
-        <v>10631.764214562814</v>
+        <v>11117.344618658306</v>
       </c>
       <c r="AK8" s="5">
         <f t="shared" ref="AK8:AO8" si="8">AJ8*1.03</f>
-        <v>10950.717140999699</v>
+        <v>11450.864957218055</v>
       </c>
       <c r="AL8" s="5">
         <f t="shared" si="8"/>
-        <v>11279.23865522969</v>
+        <v>11794.390905934597</v>
       </c>
       <c r="AM8" s="5">
         <f t="shared" si="8"/>
-        <v>11617.615814886582</v>
+        <v>12148.222633112635</v>
       </c>
       <c r="AN8" s="5">
         <f t="shared" si="8"/>
-        <v>11966.144289333179</v>
+        <v>12512.669312106014</v>
       </c>
       <c r="AO8" s="5">
         <f t="shared" si="8"/>
-        <v>12325.128618013174</v>
+        <v>12888.049391469194</v>
       </c>
     </row>
     <row r="9" spans="2:41" x14ac:dyDescent="0.3">
@@ -1777,8 +1791,7 @@
         <v>991</v>
       </c>
       <c r="U9" s="5">
-        <f>Q9*1.45</f>
-        <v>1045.45</v>
+        <v>1069</v>
       </c>
       <c r="V9" s="5">
         <f>R9*1.4</f>
@@ -1807,47 +1820,47 @@
       </c>
       <c r="AE9" s="5">
         <f>SUM(S9:V9)</f>
-        <v>4031.25</v>
+        <v>4054.8</v>
       </c>
       <c r="AF9" s="5">
         <f>AE9*1.18</f>
-        <v>4756.875</v>
+        <v>4784.6639999999998</v>
       </c>
       <c r="AG9" s="5">
         <f>AF9*1.09</f>
-        <v>5184.9937500000005</v>
+        <v>5215.2837600000003</v>
       </c>
       <c r="AH9" s="5">
         <f>AG9*1.06</f>
-        <v>5496.0933750000013</v>
+        <v>5528.2007856000009</v>
       </c>
       <c r="AI9" s="5">
         <f>AH9*1.04</f>
-        <v>5715.9371100000017</v>
+        <v>5749.3288170240012</v>
       </c>
       <c r="AJ9" s="5">
         <f>AI9*1.04</f>
-        <v>5944.5745944000018</v>
+        <v>5979.3019697049613</v>
       </c>
       <c r="AK9" s="5">
         <f t="shared" ref="AK9:AO9" si="9">AJ9*1.04</f>
-        <v>6182.3575781760019</v>
+        <v>6218.4740484931599</v>
       </c>
       <c r="AL9" s="5">
         <f t="shared" si="9"/>
-        <v>6429.6518813030425</v>
+        <v>6467.2130104328862</v>
       </c>
       <c r="AM9" s="5">
         <f t="shared" si="9"/>
-        <v>6686.8379565551641</v>
+        <v>6725.9015308502021</v>
       </c>
       <c r="AN9" s="5">
         <f t="shared" si="9"/>
-        <v>6954.3114748173712</v>
+        <v>6994.9375920842103</v>
       </c>
       <c r="AO9" s="5">
         <f t="shared" si="9"/>
-        <v>7232.4839338100664</v>
+        <v>7274.735095767579</v>
       </c>
     </row>
     <row r="10" spans="2:41" x14ac:dyDescent="0.3">
@@ -1910,11 +1923,10 @@
         <v>308</v>
       </c>
       <c r="U10" s="5">
-        <f t="shared" ref="U10:V10" si="10">Q10*0.98</f>
-        <v>344.96</v>
+        <v>302</v>
       </c>
       <c r="V10" s="5">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="V10" si="10">R10*0.98</f>
         <v>325.36</v>
       </c>
       <c r="Y10" s="5"/>
@@ -1934,7 +1946,7 @@
       </c>
       <c r="AE10" s="5">
         <f>SUM(S10:V10)</f>
-        <v>1294.3200000000002</v>
+        <v>1251.3600000000001</v>
       </c>
       <c r="AF10" s="5"/>
       <c r="AG10" s="5"/>
@@ -2039,43 +2051,43 @@
       </c>
       <c r="AF11" s="5">
         <f t="shared" ref="AF11:AO11" si="11">-AF3*0.002</f>
-        <v>-80.149199999999993</v>
+        <v>-83.872863600000017</v>
       </c>
       <c r="AG11" s="5">
         <f t="shared" si="11"/>
-        <v>-92.171579999999992</v>
+        <v>-96.453793140000016</v>
       </c>
       <c r="AH11" s="5">
         <f t="shared" si="11"/>
-        <v>-101.388738</v>
+        <v>-106.09917245400001</v>
       </c>
       <c r="AI11" s="5">
         <f t="shared" si="11"/>
-        <v>-110.51372442</v>
+        <v>-115.64809797486002</v>
       </c>
       <c r="AJ11" s="5">
         <f t="shared" si="11"/>
-        <v>-118.24968512940001</v>
+        <v>-123.74346483310023</v>
       </c>
       <c r="AK11" s="5">
         <f t="shared" si="11"/>
-        <v>-124.16216938587002</v>
+        <v>-129.93063807475525</v>
       </c>
       <c r="AL11" s="5">
         <f t="shared" si="11"/>
-        <v>-130.37027785516352</v>
+        <v>-136.42716997849303</v>
       </c>
       <c r="AM11" s="5">
         <f t="shared" si="11"/>
-        <v>-136.88879174792172</v>
+        <v>-143.24852847741766</v>
       </c>
       <c r="AN11" s="5">
         <f t="shared" si="11"/>
-        <v>-143.73323133531781</v>
+        <v>-150.41095490128856</v>
       </c>
       <c r="AO11" s="5">
         <f t="shared" si="11"/>
-        <v>-150.91989290208369</v>
+        <v>-157.93150264635298</v>
       </c>
     </row>
     <row r="12" spans="2:41" x14ac:dyDescent="0.3">
@@ -2214,11 +2226,11 @@
       </c>
       <c r="U13" s="5">
         <f t="shared" si="13"/>
-        <v>3386.33</v>
+        <v>3510</v>
       </c>
       <c r="V13" s="5">
         <f t="shared" si="13"/>
-        <v>3488.56</v>
+        <v>3625.52</v>
       </c>
       <c r="Y13" s="5">
         <f t="shared" ref="Y13:AC13" si="14">SUM(Y8:Y11)</f>
@@ -2246,47 +2258,47 @@
       </c>
       <c r="AE13" s="5">
         <f t="shared" ref="AE13:AO13" si="15">SUM(AE8:AE12)</f>
-        <v>12997.89</v>
+        <v>13258.52</v>
       </c>
       <c r="AF13" s="5">
         <f t="shared" si="15"/>
-        <v>13346.447399999999</v>
+        <v>13766.481536400001</v>
       </c>
       <c r="AG13" s="5">
         <f t="shared" si="15"/>
-        <v>14456.121497999999</v>
+        <v>14909.77559886</v>
       </c>
       <c r="AH13" s="5">
         <f t="shared" si="15"/>
-        <v>15319.801924680001</v>
+        <v>15800.503983066003</v>
       </c>
       <c r="AI13" s="5">
         <f t="shared" si="15"/>
-        <v>15927.5245647672</v>
+        <v>16427.219183765941</v>
       </c>
       <c r="AJ13" s="5">
         <f t="shared" si="15"/>
-        <v>16458.089123833415</v>
+        <v>16972.903123530166</v>
       </c>
       <c r="AK13" s="5">
         <f t="shared" si="15"/>
-        <v>17008.912549789831</v>
+        <v>17539.408367636461</v>
       </c>
       <c r="AL13" s="5">
         <f t="shared" si="15"/>
-        <v>17578.52025867757</v>
+        <v>18125.176746388992</v>
       </c>
       <c r="AM13" s="5">
         <f t="shared" si="15"/>
-        <v>18167.564979693823</v>
+        <v>18730.875635485416</v>
       </c>
       <c r="AN13" s="5">
         <f t="shared" si="15"/>
-        <v>18776.722532815231</v>
+        <v>19357.195949288933</v>
       </c>
       <c r="AO13" s="5">
         <f t="shared" si="15"/>
-        <v>19406.692658921158</v>
+        <v>20004.85298459042</v>
       </c>
     </row>
     <row r="14" spans="2:41" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2367,11 +2379,11 @@
       </c>
       <c r="U14" s="8">
         <f t="shared" si="17"/>
-        <v>1224.67</v>
+        <v>1270</v>
       </c>
       <c r="V14" s="8">
         <f t="shared" si="17"/>
-        <v>1680.5900000000006</v>
+        <v>1674.9647</v>
       </c>
       <c r="Y14" s="8">
         <f t="shared" ref="Y14:AD14" si="18">Y7-Y13</f>
@@ -2399,47 +2411,47 @@
       </c>
       <c r="AE14" s="8">
         <f t="shared" ref="AE14:AO14" si="19">AE7-AE13</f>
-        <v>3577.260000000002</v>
+        <v>3616.9647000000041</v>
       </c>
       <c r="AF14" s="8">
         <f t="shared" si="19"/>
-        <v>8694.5826000000034</v>
+        <v>9298.5559536000055</v>
       </c>
       <c r="AG14" s="8">
         <f t="shared" si="19"/>
-        <v>11812.778801999995</v>
+        <v>12579.555446040002</v>
       </c>
       <c r="AH14" s="8">
         <f t="shared" si="19"/>
-        <v>14589.875785319995</v>
+        <v>14968.256028593998</v>
       </c>
       <c r="AI14" s="8">
         <f t="shared" si="19"/>
-        <v>17226.592761232801</v>
+        <v>17688.969718817767</v>
       </c>
       <c r="AJ14" s="8">
         <f t="shared" si="19"/>
-        <v>19608.064840633589</v>
+        <v>20150.136326399901</v>
       </c>
       <c r="AK14" s="8">
         <f t="shared" si="19"/>
-        <v>21481.359959829872</v>
+        <v>21439.78305479011</v>
       </c>
       <c r="AL14" s="8">
         <f t="shared" si="19"/>
-        <v>22836.265876423124</v>
+        <v>22802.974247158912</v>
       </c>
       <c r="AM14" s="8">
         <f t="shared" si="19"/>
-        <v>24267.9604621619</v>
+        <v>24243.682907739876</v>
       </c>
       <c r="AN14" s="8">
         <f t="shared" si="19"/>
-        <v>25780.579181133286</v>
+        <v>25766.090521097631</v>
       </c>
       <c r="AO14" s="8">
         <f t="shared" si="19"/>
-        <v>27378.474140724786</v>
+        <v>27374.59780931547</v>
       </c>
     </row>
     <row r="15" spans="2:41" x14ac:dyDescent="0.3">
@@ -2502,7 +2514,7 @@
         <v>38</v>
       </c>
       <c r="U15" s="5">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="V15" s="5">
         <v>22</v>
@@ -2530,47 +2542,47 @@
       </c>
       <c r="AE15" s="5">
         <f>SUM(S15:V15)</f>
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="AF15" s="5">
         <f t="shared" ref="AF15:AO15" si="20">AE15*1.02</f>
-        <v>104.04</v>
+        <v>119.34</v>
       </c>
       <c r="AG15" s="5">
         <f t="shared" si="20"/>
-        <v>106.1208</v>
+        <v>121.72680000000001</v>
       </c>
       <c r="AH15" s="5">
         <f t="shared" si="20"/>
-        <v>108.243216</v>
+        <v>124.16133600000002</v>
       </c>
       <c r="AI15" s="5">
         <f t="shared" si="20"/>
-        <v>110.40808032000001</v>
+        <v>126.64456272000002</v>
       </c>
       <c r="AJ15" s="5">
         <f t="shared" si="20"/>
-        <v>112.61624192640001</v>
+        <v>129.17745397440004</v>
       </c>
       <c r="AK15" s="5">
         <f t="shared" si="20"/>
-        <v>114.868566764928</v>
+        <v>131.76100305388803</v>
       </c>
       <c r="AL15" s="5">
         <f t="shared" si="20"/>
-        <v>117.16593810022657</v>
+        <v>134.39622311496581</v>
       </c>
       <c r="AM15" s="5">
         <f t="shared" si="20"/>
-        <v>119.5092568622311</v>
+        <v>137.08414757726513</v>
       </c>
       <c r="AN15" s="5">
         <f t="shared" si="20"/>
-        <v>121.89944199947573</v>
+        <v>139.82583052881043</v>
       </c>
       <c r="AO15" s="5">
         <f t="shared" si="20"/>
-        <v>124.33743083946524</v>
+        <v>142.62234713938665</v>
       </c>
     </row>
     <row r="16" spans="2:41" x14ac:dyDescent="0.3">
@@ -2633,7 +2645,7 @@
         <v>-98</v>
       </c>
       <c r="U16" s="5">
-        <v>-45</v>
+        <v>-82</v>
       </c>
       <c r="V16" s="5">
         <v>-45</v>
@@ -2661,47 +2673,47 @@
       </c>
       <c r="AE16" s="5">
         <f>SUM(S16:V16)</f>
-        <v>-227</v>
+        <v>-264</v>
       </c>
       <c r="AF16" s="5">
         <f t="shared" ref="AF16:AO16" si="21">AE16*1.01</f>
-        <v>-229.27</v>
+        <v>-266.64</v>
       </c>
       <c r="AG16" s="5">
         <f t="shared" si="21"/>
-        <v>-231.56270000000001</v>
+        <v>-269.3064</v>
       </c>
       <c r="AH16" s="5">
         <f t="shared" si="21"/>
-        <v>-233.87832700000001</v>
+        <v>-271.99946399999999</v>
       </c>
       <c r="AI16" s="5">
         <f t="shared" si="21"/>
-        <v>-236.21711027000001</v>
+        <v>-274.71945863999997</v>
       </c>
       <c r="AJ16" s="5">
         <f t="shared" si="21"/>
-        <v>-238.5792813727</v>
+        <v>-277.46665322639996</v>
       </c>
       <c r="AK16" s="5">
         <f t="shared" si="21"/>
-        <v>-240.96507418642699</v>
+        <v>-280.24131975866396</v>
       </c>
       <c r="AL16" s="5">
         <f t="shared" si="21"/>
-        <v>-243.37472492829127</v>
+        <v>-283.04373295625061</v>
       </c>
       <c r="AM16" s="5">
         <f t="shared" si="21"/>
-        <v>-245.80847217757417</v>
+        <v>-285.87417028581314</v>
       </c>
       <c r="AN16" s="5">
         <f t="shared" si="21"/>
-        <v>-248.26655689934992</v>
+        <v>-288.73291198867128</v>
       </c>
       <c r="AO16" s="5">
         <f t="shared" si="21"/>
-        <v>-250.74922246834342</v>
+        <v>-291.62024110855799</v>
       </c>
     </row>
     <row r="17" spans="2:142" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2782,11 +2794,11 @@
       </c>
       <c r="U17" s="8">
         <f t="shared" si="22"/>
-        <v>1247.67</v>
+        <v>1315</v>
       </c>
       <c r="V17" s="8">
         <f t="shared" si="22"/>
-        <v>1703.5900000000006</v>
+        <v>1697.9647</v>
       </c>
       <c r="Y17" s="8">
         <f t="shared" ref="Y17:AD17" si="23">Y14-SUM(Y15:Y16)</f>
@@ -2814,47 +2826,47 @@
       </c>
       <c r="AE17" s="8">
         <f t="shared" ref="AE17:AO17" si="24">AE14-SUM(AE15:AE16)</f>
-        <v>3702.260000000002</v>
+        <v>3763.9647000000041</v>
       </c>
       <c r="AF17" s="8">
         <f t="shared" si="24"/>
-        <v>8819.8126000000029</v>
+        <v>9445.8559536000048</v>
       </c>
       <c r="AG17" s="8">
         <f t="shared" si="24"/>
-        <v>11938.220701999995</v>
+        <v>12727.135046040001</v>
       </c>
       <c r="AH17" s="8">
         <f t="shared" si="24"/>
-        <v>14715.510896319995</v>
+        <v>15116.094156593997</v>
       </c>
       <c r="AI17" s="8">
         <f t="shared" si="24"/>
-        <v>17352.401791182801</v>
+        <v>17837.044614737766</v>
       </c>
       <c r="AJ17" s="8">
         <f t="shared" si="24"/>
-        <v>19734.027880079888</v>
+        <v>20298.425525651903</v>
       </c>
       <c r="AK17" s="8">
         <f t="shared" si="24"/>
-        <v>21607.45646725137</v>
+        <v>21588.263371494886</v>
       </c>
       <c r="AL17" s="8">
         <f t="shared" si="24"/>
-        <v>22962.474663251189</v>
+        <v>22951.621757000197</v>
       </c>
       <c r="AM17" s="8">
         <f t="shared" si="24"/>
-        <v>24394.259677477243</v>
+        <v>24392.472930448424</v>
       </c>
       <c r="AN17" s="8">
         <f t="shared" si="24"/>
-        <v>25906.946296033158</v>
+        <v>25914.997602557491</v>
       </c>
       <c r="AO17" s="8">
         <f t="shared" si="24"/>
-        <v>27504.885932353664</v>
+        <v>27523.595703284642</v>
       </c>
     </row>
     <row r="18" spans="2:142" x14ac:dyDescent="0.3">
@@ -2917,12 +2929,11 @@
         <v>-834</v>
       </c>
       <c r="U18" s="5">
-        <f t="shared" ref="U18:V18" si="25">U17*0.18</f>
-        <v>224.5806</v>
+        <v>153</v>
       </c>
       <c r="V18" s="5">
-        <f t="shared" si="25"/>
-        <v>306.64620000000008</v>
+        <f t="shared" ref="V18" si="25">V17*0.18</f>
+        <v>305.633646</v>
       </c>
       <c r="Y18" s="5">
         <v>31</v>
@@ -2947,47 +2958,47 @@
       </c>
       <c r="AE18" s="5">
         <f>SUM(S18:V18)</f>
-        <v>-179.77319999999992</v>
+        <v>-252.366354</v>
       </c>
       <c r="AF18" s="5">
         <f t="shared" ref="AF18:AO18" si="26">AF17*0.12</f>
-        <v>1058.3775120000003</v>
+        <v>1133.5027144320006</v>
       </c>
       <c r="AG18" s="5">
         <f t="shared" si="26"/>
-        <v>1432.5864842399994</v>
+        <v>1527.2562055248</v>
       </c>
       <c r="AH18" s="5">
         <f t="shared" si="26"/>
-        <v>1765.8613075583992</v>
+        <v>1813.9312987912797</v>
       </c>
       <c r="AI18" s="5">
         <f t="shared" si="26"/>
-        <v>2082.2882149419361</v>
+        <v>2140.4453537685317</v>
       </c>
       <c r="AJ18" s="5">
         <f t="shared" si="26"/>
-        <v>2368.0833456095866</v>
+        <v>2435.811063078228</v>
       </c>
       <c r="AK18" s="5">
         <f t="shared" si="26"/>
-        <v>2592.8947760701644</v>
+        <v>2590.5916045793861</v>
       </c>
       <c r="AL18" s="5">
         <f t="shared" si="26"/>
-        <v>2755.4969595901425</v>
+        <v>2754.1946108400234</v>
       </c>
       <c r="AM18" s="5">
         <f t="shared" si="26"/>
-        <v>2927.3111612972689</v>
+        <v>2927.0967516538108</v>
       </c>
       <c r="AN18" s="5">
         <f t="shared" si="26"/>
-        <v>3108.8335555239787</v>
+        <v>3109.799712306899</v>
       </c>
       <c r="AO18" s="5">
         <f t="shared" si="26"/>
-        <v>3300.5863118824395</v>
+        <v>3302.8314843941571</v>
       </c>
     </row>
     <row r="19" spans="2:142" x14ac:dyDescent="0.3">
@@ -3050,12 +3061,11 @@
         <v>-8</v>
       </c>
       <c r="U19" s="5">
-        <f t="shared" ref="U19:V19" si="27">-U17*0.01</f>
-        <v>-12.476700000000001</v>
+        <v>-10</v>
       </c>
       <c r="V19" s="5">
-        <f t="shared" si="27"/>
-        <v>-17.035900000000005</v>
+        <f t="shared" ref="V19" si="27">-V17*0.01</f>
+        <v>-16.979647</v>
       </c>
       <c r="Y19" s="5">
         <v>0</v>
@@ -3080,47 +3090,47 @@
       </c>
       <c r="AE19" s="5">
         <f>SUM(S19:V19)</f>
-        <v>-44.512600000000006</v>
+        <v>-41.979647</v>
       </c>
       <c r="AF19" s="5">
         <f>-AF17*0.01</f>
-        <v>-88.19812600000003</v>
+        <v>-94.458559536000053</v>
       </c>
       <c r="AG19" s="5">
         <f t="shared" ref="AG19:AO19" si="28">-AG17*0.01</f>
-        <v>-119.38220701999995</v>
+        <v>-127.27135046040001</v>
       </c>
       <c r="AH19" s="5">
         <f t="shared" si="28"/>
-        <v>-147.15510896319995</v>
+        <v>-151.16094156593996</v>
       </c>
       <c r="AI19" s="5">
         <f t="shared" si="28"/>
-        <v>-173.52401791182803</v>
+        <v>-178.37044614737766</v>
       </c>
       <c r="AJ19" s="5">
         <f t="shared" si="28"/>
-        <v>-197.34027880079887</v>
+        <v>-202.98425525651902</v>
       </c>
       <c r="AK19" s="5">
         <f t="shared" si="28"/>
-        <v>-216.0745646725137</v>
+        <v>-215.88263371494887</v>
       </c>
       <c r="AL19" s="5">
         <f t="shared" si="28"/>
-        <v>-229.62474663251189</v>
+        <v>-229.51621757000197</v>
       </c>
       <c r="AM19" s="5">
         <f t="shared" si="28"/>
-        <v>-243.94259677477243</v>
+        <v>-243.92472930448426</v>
       </c>
       <c r="AN19" s="5">
         <f t="shared" si="28"/>
-        <v>-259.06946296033158</v>
+        <v>-259.14997602557492</v>
       </c>
       <c r="AO19" s="5">
         <f t="shared" si="28"/>
-        <v>-275.04885932353665</v>
+        <v>-275.23595703284644</v>
       </c>
     </row>
     <row r="20" spans="2:142" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -3201,11 +3211,11 @@
       </c>
       <c r="U20" s="8">
         <f t="shared" si="30"/>
-        <v>1035.5661</v>
+        <v>1172</v>
       </c>
       <c r="V20" s="8">
         <f t="shared" si="30"/>
-        <v>1413.9797000000005</v>
+        <v>1409.3107009999999</v>
       </c>
       <c r="Y20" s="8">
         <f t="shared" ref="Y20:AD20" si="31">Y17-Y18-Y19</f>
@@ -3233,451 +3243,451 @@
       </c>
       <c r="AE20" s="8">
         <f t="shared" ref="AE20:AO20" si="32">AE17-AE18-AE19</f>
-        <v>3926.5458000000021</v>
+        <v>4058.310701000004</v>
       </c>
       <c r="AF20" s="8">
         <f t="shared" si="32"/>
-        <v>7849.6332140000031</v>
+        <v>8406.8117987040041</v>
       </c>
       <c r="AG20" s="8">
         <f t="shared" si="32"/>
-        <v>10625.016424779997</v>
+        <v>11327.150190975601</v>
       </c>
       <c r="AH20" s="8">
         <f t="shared" si="32"/>
-        <v>13096.804697724794</v>
+        <v>13453.323799368658</v>
       </c>
       <c r="AI20" s="8">
         <f t="shared" si="32"/>
-        <v>15443.637594152693</v>
+        <v>15874.969707116612</v>
       </c>
       <c r="AJ20" s="8">
         <f t="shared" si="32"/>
-        <v>17563.284813271101</v>
+        <v>18065.598717830195</v>
       </c>
       <c r="AK20" s="8">
         <f t="shared" si="32"/>
-        <v>19230.636255853722</v>
+        <v>19213.554400630448</v>
       </c>
       <c r="AL20" s="8">
         <f t="shared" si="32"/>
-        <v>20436.602450293558</v>
+        <v>20426.943363730177</v>
       </c>
       <c r="AM20" s="8">
         <f t="shared" si="32"/>
-        <v>21710.891112954749</v>
+        <v>21709.300908099096</v>
       </c>
       <c r="AN20" s="8">
         <f t="shared" si="32"/>
-        <v>23057.182203469511</v>
+        <v>23064.347866276166</v>
       </c>
       <c r="AO20" s="8">
         <f t="shared" si="32"/>
-        <v>24479.34847979476</v>
+        <v>24496.000175923335</v>
       </c>
       <c r="AP20" s="3">
         <f>AO20*(1+$AR$25)</f>
-        <v>24234.554994996812</v>
+        <v>24251.0401741641</v>
       </c>
       <c r="AQ20" s="3">
         <f t="shared" ref="AQ20:DB20" si="33">AP20*(1+$AR$25)</f>
-        <v>23992.209445046843</v>
+        <v>24008.529772422458</v>
       </c>
       <c r="AR20" s="3">
         <f t="shared" si="33"/>
-        <v>23752.287350596376</v>
+        <v>23768.444474698234</v>
       </c>
       <c r="AS20" s="3">
         <f t="shared" si="33"/>
-        <v>23514.764477090412</v>
+        <v>23530.760029951252</v>
       </c>
       <c r="AT20" s="3">
         <f t="shared" si="33"/>
-        <v>23279.616832319509</v>
+        <v>23295.452429651741</v>
       </c>
       <c r="AU20" s="3">
         <f t="shared" si="33"/>
-        <v>23046.820663996314</v>
+        <v>23062.497905355223</v>
       </c>
       <c r="AV20" s="3">
         <f t="shared" si="33"/>
-        <v>22816.352457356352</v>
+        <v>22831.872926301672</v>
       </c>
       <c r="AW20" s="3">
         <f t="shared" si="33"/>
-        <v>22588.188932782788</v>
+        <v>22603.554197038655</v>
       </c>
       <c r="AX20" s="3">
         <f t="shared" si="33"/>
-        <v>22362.307043454959</v>
+        <v>22377.518655068267</v>
       </c>
       <c r="AY20" s="3">
         <f t="shared" si="33"/>
-        <v>22138.683973020408</v>
+        <v>22153.743468517583</v>
       </c>
       <c r="AZ20" s="3">
         <f t="shared" si="33"/>
-        <v>21917.297133290205</v>
+        <v>21932.206033832408</v>
       </c>
       <c r="BA20" s="3">
         <f t="shared" si="33"/>
-        <v>21698.124161957305</v>
+        <v>21712.883973494085</v>
       </c>
       <c r="BB20" s="3">
         <f t="shared" si="33"/>
-        <v>21481.14292033773</v>
+        <v>21495.755133759143</v>
       </c>
       <c r="BC20" s="3">
         <f t="shared" si="33"/>
-        <v>21266.331491134351</v>
+        <v>21280.79758242155</v>
       </c>
       <c r="BD20" s="3">
         <f t="shared" si="33"/>
-        <v>21053.668176223007</v>
+        <v>21067.989606597333</v>
       </c>
       <c r="BE20" s="3">
         <f t="shared" si="33"/>
-        <v>20843.131494460777</v>
+        <v>20857.309710531361</v>
       </c>
       <c r="BF20" s="3">
         <f t="shared" si="33"/>
-        <v>20634.700179516167</v>
+        <v>20648.736613426048</v>
       </c>
       <c r="BG20" s="3">
         <f t="shared" si="33"/>
-        <v>20428.353177721005</v>
+        <v>20442.249247291787</v>
       </c>
       <c r="BH20" s="3">
         <f t="shared" si="33"/>
-        <v>20224.069645943793</v>
+        <v>20237.826754818871</v>
       </c>
       <c r="BI20" s="3">
         <f t="shared" si="33"/>
-        <v>20021.828949484356</v>
+        <v>20035.448487270682</v>
       </c>
       <c r="BJ20" s="3">
         <f t="shared" si="33"/>
-        <v>19821.61065998951</v>
+        <v>19835.094002397975</v>
       </c>
       <c r="BK20" s="3">
         <f t="shared" si="33"/>
-        <v>19623.394553389615</v>
+        <v>19636.743062373997</v>
       </c>
       <c r="BL20" s="3">
         <f t="shared" si="33"/>
-        <v>19427.16060785572</v>
+        <v>19440.375631750256</v>
       </c>
       <c r="BM20" s="3">
         <f t="shared" si="33"/>
-        <v>19232.889001777163</v>
+        <v>19245.971875432751</v>
       </c>
       <c r="BN20" s="3">
         <f t="shared" si="33"/>
-        <v>19040.560111759391</v>
+        <v>19053.512156678426</v>
       </c>
       <c r="BO20" s="3">
         <f t="shared" si="33"/>
-        <v>18850.154510641798</v>
+        <v>18862.977035111642</v>
       </c>
       <c r="BP20" s="3">
         <f t="shared" si="33"/>
-        <v>18661.652965535381</v>
+        <v>18674.347264760527</v>
       </c>
       <c r="BQ20" s="3">
         <f t="shared" si="33"/>
-        <v>18475.036435880025</v>
+        <v>18487.603792112921</v>
       </c>
       <c r="BR20" s="3">
         <f t="shared" si="33"/>
-        <v>18290.286071521226</v>
+        <v>18302.72775419179</v>
       </c>
       <c r="BS20" s="3">
         <f t="shared" si="33"/>
-        <v>18107.383210806012</v>
+        <v>18119.700476649872</v>
       </c>
       <c r="BT20" s="3">
         <f t="shared" si="33"/>
-        <v>17926.309378697952</v>
+        <v>17938.503471883374</v>
       </c>
       <c r="BU20" s="3">
         <f t="shared" si="33"/>
-        <v>17747.046284910972</v>
+        <v>17759.11843716454</v>
       </c>
       <c r="BV20" s="3">
         <f t="shared" si="33"/>
-        <v>17569.575822061863</v>
+        <v>17581.527252792894</v>
       </c>
       <c r="BW20" s="3">
         <f t="shared" si="33"/>
-        <v>17393.880063841243</v>
+        <v>17405.711980264965</v>
       </c>
       <c r="BX20" s="3">
         <f t="shared" si="33"/>
-        <v>17219.941263202829</v>
+        <v>17231.654860462317</v>
       </c>
       <c r="BY20" s="3">
         <f t="shared" si="33"/>
-        <v>17047.741850570801</v>
+        <v>17059.338311857693</v>
       </c>
       <c r="BZ20" s="3">
         <f t="shared" si="33"/>
-        <v>16877.264432065094</v>
+        <v>16888.744928739117</v>
       </c>
       <c r="CA20" s="3">
         <f t="shared" si="33"/>
-        <v>16708.491787744442</v>
+        <v>16719.857479451726</v>
       </c>
       <c r="CB20" s="3">
         <f t="shared" si="33"/>
-        <v>16541.406869866998</v>
+        <v>16552.658904657208</v>
       </c>
       <c r="CC20" s="3">
         <f t="shared" si="33"/>
-        <v>16375.992801168328</v>
+        <v>16387.132315610637</v>
       </c>
       <c r="CD20" s="3">
         <f t="shared" si="33"/>
-        <v>16212.232873156645</v>
+        <v>16223.26099245453</v>
       </c>
       <c r="CE20" s="3">
         <f t="shared" si="33"/>
-        <v>16050.110544425079</v>
+        <v>16061.028382529985</v>
       </c>
       <c r="CF20" s="3">
         <f t="shared" si="33"/>
-        <v>15889.609438980828</v>
+        <v>15900.418098704686</v>
       </c>
       <c r="CG20" s="3">
         <f t="shared" si="33"/>
-        <v>15730.713344591019</v>
+        <v>15741.413917717638</v>
       </c>
       <c r="CH20" s="3">
         <f t="shared" si="33"/>
-        <v>15573.406211145108</v>
+        <v>15583.999778540461</v>
       </c>
       <c r="CI20" s="3">
         <f t="shared" si="33"/>
-        <v>15417.672149033657</v>
+        <v>15428.159780755057</v>
       </c>
       <c r="CJ20" s="3">
         <f t="shared" si="33"/>
-        <v>15263.495427543319</v>
+        <v>15273.878182947507</v>
       </c>
       <c r="CK20" s="3">
         <f t="shared" si="33"/>
-        <v>15110.860473267885</v>
+        <v>15121.139401118031</v>
       </c>
       <c r="CL20" s="3">
         <f t="shared" si="33"/>
-        <v>14959.751868535206</v>
+        <v>14969.92800710685</v>
       </c>
       <c r="CM20" s="3">
         <f t="shared" si="33"/>
-        <v>14810.154349849854</v>
+        <v>14820.228727035781</v>
       </c>
       <c r="CN20" s="3">
         <f t="shared" si="33"/>
-        <v>14662.052806351356</v>
+        <v>14672.026439765423</v>
       </c>
       <c r="CO20" s="3">
         <f t="shared" si="33"/>
-        <v>14515.432278287843</v>
+        <v>14525.306175367768</v>
       </c>
       <c r="CP20" s="3">
         <f t="shared" si="33"/>
-        <v>14370.277955504964</v>
+        <v>14380.053113614091</v>
       </c>
       <c r="CQ20" s="3">
         <f t="shared" si="33"/>
-        <v>14226.575175949914</v>
+        <v>14236.25258247795</v>
       </c>
       <c r="CR20" s="3">
         <f t="shared" si="33"/>
-        <v>14084.309424190415</v>
+        <v>14093.89005665317</v>
       </c>
       <c r="CS20" s="3">
         <f t="shared" si="33"/>
-        <v>13943.466329948511</v>
+        <v>13952.951156086638</v>
       </c>
       <c r="CT20" s="3">
         <f t="shared" si="33"/>
-        <v>13804.031666649025</v>
+        <v>13813.421644525772</v>
       </c>
       <c r="CU20" s="3">
         <f t="shared" si="33"/>
-        <v>13665.991349982534</v>
+        <v>13675.287428080514</v>
       </c>
       <c r="CV20" s="3">
         <f t="shared" si="33"/>
-        <v>13529.331436482709</v>
+        <v>13538.534553799709</v>
       </c>
       <c r="CW20" s="3">
         <f t="shared" si="33"/>
-        <v>13394.038122117881</v>
+        <v>13403.149208261711</v>
       </c>
       <c r="CX20" s="3">
         <f t="shared" si="33"/>
-        <v>13260.097740896703</v>
+        <v>13269.117716179095</v>
       </c>
       <c r="CY20" s="3">
         <f t="shared" si="33"/>
-        <v>13127.496763487736</v>
+        <v>13136.426539017304</v>
       </c>
       <c r="CZ20" s="3">
         <f t="shared" si="33"/>
-        <v>12996.221795852858</v>
+        <v>13005.062273627131</v>
       </c>
       <c r="DA20" s="3">
         <f t="shared" si="33"/>
-        <v>12866.259577894329</v>
+        <v>12875.01165089086</v>
       </c>
       <c r="DB20" s="3">
         <f t="shared" si="33"/>
-        <v>12737.596982115385</v>
+        <v>12746.261534381951</v>
       </c>
       <c r="DC20" s="3">
         <f t="shared" ref="DC20:EL20" si="34">DB20*(1+$AR$25)</f>
-        <v>12610.221012294231</v>
+        <v>12618.79891903813</v>
       </c>
       <c r="DD20" s="3">
         <f t="shared" si="34"/>
-        <v>12484.118802171288</v>
+        <v>12492.61092984775</v>
       </c>
       <c r="DE20" s="3">
         <f t="shared" si="34"/>
-        <v>12359.277614149574</v>
+        <v>12367.684820549272</v>
       </c>
       <c r="DF20" s="3">
         <f t="shared" si="34"/>
-        <v>12235.684838008079</v>
+        <v>12244.007972343779</v>
       </c>
       <c r="DG20" s="3">
         <f t="shared" si="34"/>
-        <v>12113.327989627998</v>
+        <v>12121.567892620342</v>
       </c>
       <c r="DH20" s="3">
         <f t="shared" si="34"/>
-        <v>11992.194709731719</v>
+        <v>12000.352213694137</v>
       </c>
       <c r="DI20" s="3">
         <f t="shared" si="34"/>
-        <v>11872.272762634402</v>
+        <v>11880.348691557196</v>
       </c>
       <c r="DJ20" s="3">
         <f t="shared" si="34"/>
-        <v>11753.550035008058</v>
+        <v>11761.545204641623</v>
       </c>
       <c r="DK20" s="3">
         <f t="shared" si="34"/>
-        <v>11636.014534657977</v>
+        <v>11643.929752595206</v>
       </c>
       <c r="DL20" s="3">
         <f t="shared" si="34"/>
-        <v>11519.654389311398</v>
+        <v>11527.490455069254</v>
       </c>
       <c r="DM20" s="3">
         <f t="shared" si="34"/>
-        <v>11404.457845418283</v>
+        <v>11412.21555051856</v>
       </c>
       <c r="DN20" s="3">
         <f t="shared" si="34"/>
-        <v>11290.4132669641</v>
+        <v>11298.093395013375</v>
       </c>
       <c r="DO20" s="3">
         <f t="shared" si="34"/>
-        <v>11177.50913429446</v>
+        <v>11185.112461063241</v>
       </c>
       <c r="DP20" s="3">
         <f t="shared" si="34"/>
-        <v>11065.734042951515</v>
+        <v>11073.26133645261</v>
       </c>
       <c r="DQ20" s="3">
         <f t="shared" si="34"/>
-        <v>10955.076702521999</v>
+        <v>10962.528723088084</v>
       </c>
       <c r="DR20" s="3">
         <f t="shared" si="34"/>
-        <v>10845.525935496778</v>
+        <v>10852.903435857203</v>
       </c>
       <c r="DS20" s="3">
         <f t="shared" si="34"/>
-        <v>10737.070676141811</v>
+        <v>10744.37440149863</v>
       </c>
       <c r="DT20" s="3">
         <f t="shared" si="34"/>
-        <v>10629.699969380394</v>
+        <v>10636.930657483643</v>
       </c>
       <c r="DU20" s="3">
         <f t="shared" si="34"/>
-        <v>10523.402969686589</v>
+        <v>10530.561350908807</v>
       </c>
       <c r="DV20" s="3">
         <f t="shared" si="34"/>
-        <v>10418.168939989722</v>
+        <v>10425.255737399719</v>
       </c>
       <c r="DW20" s="3">
         <f t="shared" si="34"/>
-        <v>10313.987250589826</v>
+        <v>10321.003180025722</v>
       </c>
       <c r="DX20" s="3">
         <f t="shared" si="34"/>
-        <v>10210.847378083927</v>
+        <v>10217.793148225464</v>
       </c>
       <c r="DY20" s="3">
         <f t="shared" si="34"/>
-        <v>10108.738904303087</v>
+        <v>10115.61521674321</v>
       </c>
       <c r="DZ20" s="3">
         <f t="shared" si="34"/>
-        <v>10007.651515260057</v>
+        <v>10014.459064575778</v>
       </c>
       <c r="EA20" s="3">
         <f t="shared" si="34"/>
-        <v>9907.5750001074557</v>
+        <v>9914.3144739300205</v>
       </c>
       <c r="EB20" s="3">
         <f t="shared" si="34"/>
-        <v>9808.4992501063807</v>
+        <v>9815.1713291907199</v>
       </c>
       <c r="EC20" s="3">
         <f t="shared" si="34"/>
-        <v>9710.4142576053164</v>
+        <v>9717.0196158988128</v>
       </c>
       <c r="ED20" s="3">
         <f t="shared" si="34"/>
-        <v>9613.3101150292623</v>
+        <v>9619.849419739825</v>
       </c>
       <c r="EE20" s="3">
         <f t="shared" si="34"/>
-        <v>9517.1770138789689</v>
+        <v>9523.6509255424262</v>
       </c>
       <c r="EF20" s="3">
         <f t="shared" si="34"/>
-        <v>9422.0052437401791</v>
+        <v>9428.4144162870016</v>
       </c>
       <c r="EG20" s="3">
         <f t="shared" si="34"/>
-        <v>9327.7851913027771</v>
+        <v>9334.1302721241318</v>
       </c>
       <c r="EH20" s="3">
         <f t="shared" si="34"/>
-        <v>9234.5073393897492</v>
+        <v>9240.7889694028909</v>
       </c>
       <c r="EI20" s="3">
         <f t="shared" si="34"/>
-        <v>9142.1622659958521</v>
+        <v>9148.3810797088627</v>
       </c>
       <c r="EJ20" s="3">
         <f t="shared" si="34"/>
-        <v>9050.7406433358938</v>
+        <v>9056.8972689117745</v>
       </c>
       <c r="EK20" s="3">
         <f t="shared" si="34"/>
-        <v>8960.2332369025353</v>
+        <v>8966.3282962226567</v>
       </c>
       <c r="EL20" s="3">
         <f t="shared" si="34"/>
-        <v>8870.6309045335092</v>
+        <v>8876.66501326043</v>
       </c>
     </row>
     <row r="21" spans="2:142" x14ac:dyDescent="0.3">
@@ -3742,12 +3752,12 @@
         <v>1623</v>
       </c>
       <c r="U21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="V21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="Y21" s="5">
         <v>1622.8</v>
@@ -3769,48 +3779,48 @@
         <v>1620.5</v>
       </c>
       <c r="AE21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AF21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AG21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AH21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AI21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AJ21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AK21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AL21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AM21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AN21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
       <c r="AO21" s="5">
-        <f>1623</f>
-        <v>1623</v>
+        <f>1626</f>
+        <v>1626</v>
       </c>
     </row>
     <row r="22" spans="2:142" x14ac:dyDescent="0.3">
@@ -3891,11 +3901,11 @@
       </c>
       <c r="U22" s="7">
         <f t="shared" si="37"/>
-        <v>0.63805674676524959</v>
+        <v>0.72078720787207873</v>
       </c>
       <c r="V22" s="7">
         <f t="shared" si="37"/>
-        <v>0.87121361675908848</v>
+        <v>0.86673474846248455</v>
       </c>
       <c r="Y22" s="7">
         <f t="shared" ref="Y22:AD22" si="38">Y20/Y21</f>
@@ -3923,47 +3933,47 @@
       </c>
       <c r="AE22" s="7">
         <f t="shared" ref="AE22:AO22" si="39">AE20/AE21</f>
-        <v>2.4193134935305003</v>
+        <v>2.4958860399754021</v>
       </c>
       <c r="AF22" s="7">
         <f t="shared" si="39"/>
-        <v>4.8364961269254483</v>
+        <v>5.1702409586125491</v>
       </c>
       <c r="AG22" s="7">
         <f t="shared" si="39"/>
-        <v>6.546528912372148</v>
+        <v>6.9662670301202958</v>
       </c>
       <c r="AH22" s="7">
         <f t="shared" si="39"/>
-        <v>8.0695038186844084</v>
+        <v>8.2738768753804788</v>
       </c>
       <c r="AI22" s="7">
         <f t="shared" si="39"/>
-        <v>9.5154883512955593</v>
+        <v>9.7632040019167352</v>
       </c>
       <c r="AJ22" s="7">
         <f t="shared" si="39"/>
-        <v>10.821494031590326</v>
+        <v>11.110454316008729</v>
       </c>
       <c r="AK22" s="7">
         <f t="shared" si="39"/>
-        <v>11.848820860045423</v>
+        <v>11.816454120928935</v>
       </c>
       <c r="AL22" s="7">
         <f t="shared" si="39"/>
-        <v>12.591868422854935</v>
+        <v>12.562695795652015</v>
       </c>
       <c r="AM22" s="7">
         <f t="shared" si="39"/>
-        <v>13.377012392455175</v>
+        <v>13.351353572016665</v>
       </c>
       <c r="AN22" s="7">
         <f t="shared" si="39"/>
-        <v>14.206520150012022</v>
+        <v>14.184715784917691</v>
       </c>
       <c r="AO22" s="7">
         <f t="shared" si="39"/>
-        <v>15.082777868018953</v>
+        <v>15.065190760100451</v>
       </c>
     </row>
     <row r="24" spans="2:142" x14ac:dyDescent="0.3">
@@ -4032,11 +4042,11 @@
       </c>
       <c r="U24" s="9">
         <f t="shared" ref="U24" si="43">U3/Q3-1</f>
-        <v>0.27584689837219534</v>
+        <v>0.35591728992520899</v>
       </c>
       <c r="V24" s="9">
         <f t="shared" ref="V24" si="44">V3/R3-1</f>
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="Y24" s="9"/>
       <c r="Z24" s="9">
@@ -4061,11 +4071,11 @@
       </c>
       <c r="AE24" s="9">
         <f t="shared" si="45"/>
-        <v>0.29515222028311028</v>
+        <v>0.32226720961799504</v>
       </c>
       <c r="AF24" s="9">
         <f t="shared" si="45"/>
-        <v>0.19999999999999996</v>
+        <v>0.22999999999999998</v>
       </c>
       <c r="AG24" s="9">
         <f t="shared" si="45"/>
@@ -4182,11 +4192,11 @@
       </c>
       <c r="U25" s="9">
         <f t="shared" si="48"/>
-        <v>0.53</v>
+        <v>0.51698031581224313</v>
       </c>
       <c r="V25" s="9">
         <f t="shared" si="48"/>
-        <v>0.54</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="Y25" s="9">
         <f t="shared" ref="Y25" si="49">Y7/Y3</f>
@@ -4214,7 +4224,7 @@
       </c>
       <c r="AE25" s="9">
         <f t="shared" si="50"/>
-        <v>0.49632884670090288</v>
+        <v>0.49495975909423945</v>
       </c>
       <c r="AF25" s="9">
         <f t="shared" si="50"/>
@@ -4226,35 +4236,35 @@
       </c>
       <c r="AH25" s="9">
         <f t="shared" si="50"/>
-        <v>0.59</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="AI25" s="9">
         <f t="shared" si="50"/>
-        <v>0.6</v>
+        <v>0.59000000000000008</v>
       </c>
       <c r="AJ25" s="9">
         <f t="shared" si="50"/>
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="AK25" s="9">
         <f t="shared" si="50"/>
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="AL25" s="9">
         <f t="shared" si="50"/>
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="AM25" s="9">
         <f t="shared" si="50"/>
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="AN25" s="9">
         <f t="shared" si="50"/>
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="AO25" s="9">
         <f t="shared" si="50"/>
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="AQ25" t="s">
         <v>54</v>
@@ -4341,18 +4351,18 @@
       </c>
       <c r="U26" s="9">
         <f t="shared" si="53"/>
-        <v>1</v>
+        <v>0.54510058403633999</v>
       </c>
       <c r="V26" s="9">
         <f t="shared" si="53"/>
-        <v>1</v>
+        <v>0.57276161206540221</v>
       </c>
       <c r="Y26" s="9">
         <f t="shared" ref="Y26" si="54">(Y3-Y4)/Y3</f>
         <v>0.42608824840291187</v>
       </c>
       <c r="Z26" s="9">
-        <f t="shared" ref="Z26:AD26" si="55">(Z3-Z4)/Z3</f>
+        <f t="shared" ref="Z26:AE26" si="55">(Z3-Z4)/Z3</f>
         <v>0.44525248386766364</v>
       </c>
       <c r="AA26" s="9">
@@ -4371,7 +4381,10 @@
         <f t="shared" si="55"/>
         <v>0.53019197207678881</v>
       </c>
-      <c r="AE26" s="9"/>
+      <c r="AE26" s="9">
+        <f t="shared" si="55"/>
+        <v>0.52549239968957029</v>
+      </c>
       <c r="AF26" s="9"/>
       <c r="AG26" s="9"/>
       <c r="AH26" s="9"/>
@@ -4455,11 +4468,11 @@
       </c>
       <c r="U27" s="9">
         <f t="shared" ref="U27:U28" si="59">U8/Q8-1</f>
-        <v>0.21999999999999997</v>
+        <v>0.30745721271393633</v>
       </c>
       <c r="V27" s="9">
         <f t="shared" ref="V27:V28" si="60">V8/R8-1</f>
-        <v>0.19999999999999996</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="Y27" s="9"/>
       <c r="Z27" s="9">
@@ -4484,11 +4497,11 @@
       </c>
       <c r="AE27" s="9">
         <f t="shared" si="61"/>
-        <v>0.18840148698884751</v>
+        <v>0.23177819083023543</v>
       </c>
       <c r="AF27" s="9">
         <f t="shared" si="61"/>
-        <v>0.12999999999999989</v>
+        <v>0.1399999999999999</v>
       </c>
       <c r="AG27" s="9">
         <f t="shared" si="61"/>
@@ -4531,7 +4544,7 @@
       </c>
       <c r="AR27" s="5">
         <f>NPV(AR26,AE20:EL20)</f>
-        <v>300334.0880058615</v>
+        <v>302620.97708222189</v>
       </c>
     </row>
     <row r="28" spans="2:142" x14ac:dyDescent="0.3">
@@ -4600,7 +4613,7 @@
       </c>
       <c r="U28" s="9">
         <f t="shared" si="59"/>
-        <v>0.44999999999999996</v>
+        <v>0.48266296809986131</v>
       </c>
       <c r="V28" s="9">
         <f t="shared" si="60"/>
@@ -4629,7 +4642,7 @@
       </c>
       <c r="AE28" s="9">
         <f t="shared" si="63"/>
-        <v>0.44852676967301464</v>
+        <v>0.4569888609414301</v>
       </c>
       <c r="AF28" s="9">
         <f t="shared" si="63"/>
@@ -4676,7 +4689,7 @@
       </c>
       <c r="AR28" s="5">
         <f>Main!D8</f>
-        <v>2649</v>
+        <v>4023</v>
       </c>
     </row>
     <row r="29" spans="2:142" x14ac:dyDescent="0.3">
@@ -4757,11 +4770,11 @@
       </c>
       <c r="U29" s="9">
         <f t="shared" si="66"/>
-        <v>0.12016666666666667</v>
+        <v>0.11561756435215229</v>
       </c>
       <c r="V29" s="9">
         <f t="shared" si="66"/>
-        <v>0.11583180987202925</v>
+        <v>0.11400768688191855</v>
       </c>
       <c r="Y29" s="9">
         <f t="shared" ref="Y29" si="67">Y9/Y3</f>
@@ -4789,54 +4802,54 @@
       </c>
       <c r="AE29" s="9">
         <f t="shared" si="68"/>
-        <v>0.12071237142728811</v>
+        <v>0.11892771477996847</v>
       </c>
       <c r="AF29" s="9">
         <f t="shared" si="68"/>
-        <v>0.11870049857016664</v>
+        <v>0.11409325482956323</v>
       </c>
       <c r="AG29" s="9">
         <f t="shared" si="68"/>
-        <v>0.11250742907954928</v>
+        <v>0.1081405632732382</v>
       </c>
       <c r="AH29" s="9">
         <f t="shared" si="68"/>
-        <v>0.10841624984029294</v>
+        <v>0.10420817915421138</v>
       </c>
       <c r="AI29" s="9">
         <f t="shared" si="68"/>
-        <v>0.10344302737055473</v>
+        <v>9.9427987449889746E-2</v>
       </c>
       <c r="AJ29" s="9">
         <f t="shared" si="68"/>
-        <v>0.10054275557511862</v>
+        <v>9.6640286867182554E-2</v>
       </c>
       <c r="AK29" s="9">
         <f t="shared" si="68"/>
-        <v>9.9585205522022241E-2</v>
+        <v>9.5719903182733199E-2</v>
       </c>
       <c r="AL29" s="9">
         <f t="shared" si="68"/>
-        <v>9.8636774993241083E-2</v>
+        <v>9.4808285057183361E-2</v>
       </c>
       <c r="AM29" s="9">
         <f t="shared" si="68"/>
-        <v>9.7697377136162597E-2</v>
+        <v>9.3905349009019715E-2</v>
       </c>
       <c r="AN29" s="9">
         <f t="shared" si="68"/>
-        <v>9.6766925925341987E-2</v>
+        <v>9.3011012351790948E-2</v>
       </c>
       <c r="AO29" s="9">
         <f t="shared" si="68"/>
-        <v>9.5845336154624455E-2</v>
+        <v>9.2125193186535795E-2</v>
       </c>
       <c r="AQ29" t="s">
         <v>58</v>
       </c>
       <c r="AR29" s="5">
         <f>AR27+AR28</f>
-        <v>302983.0880058615</v>
+        <v>306643.97708222189</v>
       </c>
     </row>
     <row r="30" spans="2:142" x14ac:dyDescent="0.3">
@@ -4917,11 +4930,11 @@
       </c>
       <c r="U30" s="9">
         <f t="shared" si="70"/>
-        <v>3.9650574712643674E-2</v>
+        <v>3.266277309106641E-2</v>
       </c>
       <c r="V30" s="9">
         <f t="shared" si="70"/>
-        <v>3.3989031078610607E-2</v>
+        <v>3.3453770746663981E-2</v>
       </c>
       <c r="Y30" s="9">
         <f t="shared" ref="Y30" si="71">Y10/Y3</f>
@@ -4949,7 +4962,7 @@
       </c>
       <c r="AE30" s="9">
         <f t="shared" si="72"/>
-        <v>3.8757317602671024E-2</v>
+        <v>3.6702521743874263E-2</v>
       </c>
       <c r="AF30" s="9"/>
       <c r="AG30" s="9"/>
@@ -4966,7 +4979,7 @@
       </c>
       <c r="AR30" s="4">
         <f>AR29/AO21</f>
-        <v>186.68089217859611</v>
+        <v>188.58793178488432</v>
       </c>
     </row>
     <row r="31" spans="2:142" x14ac:dyDescent="0.3">
@@ -5047,11 +5060,11 @@
       </c>
       <c r="U31" s="9">
         <f t="shared" si="75"/>
-        <v>0.14076666666666668</v>
+        <v>0.13735669478693488</v>
       </c>
       <c r="V31" s="9">
         <f t="shared" si="75"/>
-        <v>0.17556437712196402</v>
+        <v>0.17222118601719574</v>
       </c>
       <c r="Y31" s="9">
         <f t="shared" ref="Y31" si="76">Y14/Y3</f>
@@ -5079,54 +5092,54 @@
       </c>
       <c r="AE31" s="9">
         <f t="shared" si="77"/>
-        <v>0.10711802488359216</v>
+        <v>0.1060859589155605</v>
       </c>
       <c r="AF31" s="9">
         <f t="shared" si="77"/>
-        <v>0.21695993472174405</v>
+        <v>0.22172978373424712</v>
       </c>
       <c r="AG31" s="9">
         <f t="shared" si="77"/>
-        <v>0.25632149957720152</v>
+        <v>0.26084107294320974</v>
       </c>
       <c r="AH31" s="9">
         <f t="shared" si="77"/>
-        <v>0.28780071777439414</v>
+        <v>0.28215594301800201</v>
       </c>
       <c r="AI31" s="9">
         <f t="shared" si="77"/>
-        <v>0.3117548132893303</v>
+        <v>0.30591025755846074</v>
       </c>
       <c r="AJ31" s="9">
         <f t="shared" si="77"/>
-        <v>0.33163834337785486</v>
+        <v>0.32567596767356599</v>
       </c>
       <c r="AK31" s="9">
         <f t="shared" si="77"/>
-        <v>0.34602101535565644</v>
+        <v>0.33001889889057251</v>
       </c>
       <c r="AL31" s="9">
         <f t="shared" si="77"/>
-        <v>0.35032932739152944</v>
+        <v>0.33428787316710706</v>
       </c>
       <c r="AM31" s="9">
         <f t="shared" si="77"/>
-        <v>0.35456460901270753</v>
+        <v>0.3384842157252842</v>
       </c>
       <c r="AN31" s="9">
         <f t="shared" si="77"/>
-        <v>0.35872816524926399</v>
+        <v>0.3426092273399548</v>
       </c>
       <c r="AO31" s="9">
         <f t="shared" si="77"/>
-        <v>0.36282127709284612</v>
+        <v>0.34666418479679573</v>
       </c>
       <c r="AQ31" t="s">
         <v>60</v>
       </c>
       <c r="AR31" s="4">
         <f>Main!D3</f>
-        <v>150.74</v>
+        <v>239.23</v>
       </c>
     </row>
     <row r="32" spans="2:142" x14ac:dyDescent="0.3">
@@ -5207,7 +5220,7 @@
       </c>
       <c r="U32" s="9">
         <f t="shared" si="80"/>
-        <v>0.18</v>
+        <v>0.11634980988593156</v>
       </c>
       <c r="V32" s="9">
         <f t="shared" si="80"/>
@@ -5239,19 +5252,19 @@
       </c>
       <c r="AE32" s="9">
         <f t="shared" si="82"/>
-        <v>-4.8557691788259014E-2</v>
+        <v>-6.7048012963564649E-2</v>
       </c>
       <c r="AF32" s="9">
         <f t="shared" si="82"/>
-        <v>0.12</v>
+        <v>0.12000000000000001</v>
       </c>
       <c r="AG32" s="9">
         <f t="shared" si="82"/>
-        <v>0.12</v>
+        <v>0.11999999999999998</v>
       </c>
       <c r="AH32" s="9">
         <f t="shared" si="82"/>
-        <v>0.11999999999999998</v>
+        <v>0.12</v>
       </c>
       <c r="AI32" s="9">
         <f t="shared" si="82"/>
@@ -5259,11 +5272,11 @@
       </c>
       <c r="AJ32" s="9">
         <f t="shared" si="82"/>
-        <v>0.12</v>
+        <v>0.11999999999999998</v>
       </c>
       <c r="AK32" s="9">
         <f t="shared" si="82"/>
-        <v>0.12000000000000001</v>
+        <v>0.11999999999999998</v>
       </c>
       <c r="AL32" s="9">
         <f t="shared" si="82"/>
@@ -5275,18 +5288,18 @@
       </c>
       <c r="AN32" s="9">
         <f t="shared" si="82"/>
-        <v>0.11999999999999998</v>
+        <v>0.12000000000000001</v>
       </c>
       <c r="AO32" s="9">
         <f t="shared" si="82"/>
-        <v>0.12</v>
+        <v>0.12000000000000001</v>
       </c>
       <c r="AQ32" s="3" t="s">
         <v>61</v>
       </c>
       <c r="AR32" s="10">
         <f>AR30/AR31-1</f>
-        <v>0.2384296946968032</v>
+        <v>-0.21168778253193865</v>
       </c>
     </row>
     <row r="33" spans="2:44" x14ac:dyDescent="0.3">
@@ -5367,11 +5380,11 @@
       </c>
       <c r="U33" s="9">
         <f t="shared" si="85"/>
-        <v>0.11903058620689655</v>
+        <v>0.12675751676400607</v>
       </c>
       <c r="V33" s="9">
         <f t="shared" si="85"/>
-        <v>0.14771268738574045</v>
+        <v>0.14490643318808183</v>
       </c>
       <c r="Y33" s="9">
         <f t="shared" ref="Y33" si="86">Y20/Y3</f>
@@ -5399,53 +5412,53 @@
       </c>
       <c r="AE33" s="9">
         <f t="shared" si="87"/>
-        <v>0.1175770927220734</v>
+        <v>0.11903068401327374</v>
       </c>
       <c r="AF33" s="9">
         <f t="shared" si="87"/>
-        <v>0.19587552250053658</v>
+        <v>0.20046559609070039</v>
       </c>
       <c r="AG33" s="9">
         <f t="shared" si="87"/>
-        <v>0.23054864470762024</v>
+        <v>0.23487205266328004</v>
       </c>
       <c r="AH33" s="9">
         <f t="shared" si="87"/>
-        <v>0.25834831276280001</v>
+        <v>0.2535990335872117</v>
       </c>
       <c r="AI33" s="9">
         <f t="shared" si="87"/>
-        <v>0.27948813914659476</v>
+        <v>0.27453922693250982</v>
       </c>
       <c r="AJ33" s="9">
         <f t="shared" si="87"/>
-        <v>0.29705423391278701</v>
+        <v>0.29198469175234887</v>
       </c>
       <c r="AK33" s="9">
         <f t="shared" si="87"/>
-        <v>0.30976643451015956</v>
+        <v>0.29575094350842762</v>
       </c>
       <c r="AL33" s="9">
         <f t="shared" si="87"/>
-        <v>0.31351628279871974</v>
+        <v>0.29945564900232663</v>
       </c>
       <c r="AM33" s="9">
         <f t="shared" si="87"/>
-        <v>0.31720480304822868</v>
+        <v>0.3030998103624003</v>
       </c>
       <c r="AN33" s="9">
         <f t="shared" si="87"/>
-        <v>0.32083300416003313</v>
+        <v>0.30668441512671463</v>
       </c>
       <c r="AO33" s="9">
         <f t="shared" si="87"/>
-        <v>0.32440187981947322</v>
+        <v>0.31021043636589507</v>
       </c>
       <c r="AQ33" t="s">
         <v>62</v>
       </c>
       <c r="AR33" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>